<commit_message>
Biên bản GĐ2 lần 2: BUG_API_003 kiểm lại đạt; bỏ .env khỏi git
- BUG_API_003: token Nhà tuyển dụng gọi GET /candidate/applications nay trả 403
  INVALID_USER_TYPE -> đạt. Còn 20/21 mã chặn duyệt chưa đạt, kết luận vẫn CHƯA ĐẠT.
- Thêm .gitignore cho .env (file tài khoản demo chỉ để chạy kiểm thử cục bộ).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_019cva3M8RCprGJ5PLUwgHJy
</commit_message>
<xml_diff>
--- a/nghiem_thu_gd2/BaoCao_NghiemThu_GD2_lan2.xlsx
+++ b/nghiem_thu_gd2/BaoCao_NghiemThu_GD2_lan2.xlsx
@@ -1329,7 +1329,7 @@
       </c>
       <c r="C10" s="9" t="inlineStr">
         <is>
-          <t>Không đăng nhập được tài khoản NTD / Ứng viên: website chặn mọi API khi email chưa kích hoạt (EMAIL_NOT_VERIFIED) và chưa có hộp thư nhận email kích hoạt. Các lỗi trong khu NTD sau đăng nhập (F2–F8) chưa chạy lại được trên giao diện; được đánh giá theo trạng thái QA, kèm bằng chứng mã nguồn nếu có. Đã kiểm thật: 12 lỗi Verified ở trang công khai, Retest_BUG_028 (4G), Retest_BUG_047 và 4 lỗi API.</t>
+          <t>Đã đăng nhập được bằng tài khoản demo trong .env nhưng phần chạy lại F1–F8 và 40 lỗi Verified sau đăng nhập chưa thực hiện trong phiên này. Các lỗi đó được đánh giá theo trạng thái QA, kèm bằng chứng mã nguồn nếu có. Đã kiểm thật: 12 lỗi Verified ở trang công khai, Retest_BUG_028 (4G), Retest_BUG_047 và 4 lỗi API (BUG_API_003 bằng token NTD).</t>
         </is>
       </c>
       <c r="D10" s="10" t="n"/>
@@ -1515,13 +1515,13 @@
       </c>
       <c r="D23" s="15" t="inlineStr">
         <is>
-          <t>0/6 đạt</t>
+          <t>1/6 đạt</t>
         </is>
       </c>
       <c r="E23" s="12" t="n"/>
       <c r="F23" s="13" t="inlineStr">
         <is>
-          <t>còn mở 2, không đạt 2, chờ kiểm lại 2</t>
+          <t>không đạt 2, chờ kiểm lại 2, đã đạt 1, còn mở 1</t>
         </is>
       </c>
     </row>
@@ -1735,7 +1735,7 @@
       </c>
       <c r="C35" s="7" t="inlineStr">
         <is>
-          <t>Còn 21/21 mã chặn duyệt chưa đạt — CÒN MỞ (15): Retest_BUG_023, Retest_BUG_025, Retest_BUG_026, Retest_BUG_029, Retest_BUG_030, Retest_BUG_044, BUG_FUNC_035, BUG_FUNC_017, BUG_UI_081, BUG_UI_082, BUG_FUNC_046, BUG_FUNC_047, BUG_UI_086, BUG_API_003, BUG_FUNC_045; CHỜ KIỂM LẠI (3): Retest_BUG_027, BUG_FUNC_050, BUG_FUNC_018; KHÔNG ĐẠT (3): Retest_BUG_028, BUG_API_002, Retest_BUG_047. Bản giao diện 15/10 đã có thay đổi cho một số lỗi (xem cột Bằng chứng mã nguồn) nhưng chưa được kiểm lại trên tài khoản NTD nên chưa tính đạt. Các luồng chính vẫn chạy từ đầu đến cuối như lần 1.</t>
+          <t>Còn 20/21 mã chặn duyệt chưa đạt — CÒN MỞ (14): Retest_BUG_023, Retest_BUG_025, Retest_BUG_026, Retest_BUG_029, Retest_BUG_030, Retest_BUG_044, BUG_FUNC_035, BUG_FUNC_017, BUG_UI_081, BUG_UI_082, BUG_FUNC_046, BUG_FUNC_047, BUG_UI_086, BUG_FUNC_045; CHỜ KIỂM LẠI (3): Retest_BUG_027, BUG_FUNC_050, BUG_FUNC_018; KHÔNG ĐẠT (3): Retest_BUG_028, BUG_API_002, Retest_BUG_047. Bản giao diện 15/10 đã có thay đổi cho một số lỗi (xem cột Bằng chứng mã nguồn) nhưng chưa được kiểm lại trên tài khoản NTD nên chưa tính đạt. Các luồng chính vẫn chạy từ đầu đến cuối như lần 1.</t>
         </is>
       </c>
       <c r="D35" s="8" t="n"/>
@@ -1756,7 +1756,7 @@
     <row r="38" ht="34" customHeight="1">
       <c r="B38" s="18" t="inlineStr">
         <is>
-          <t>•  Dev sửa 21 mã chặn duyệt ở sheet "Điểm chặn", ưu tiên BUG_API_003 (token NTD đọc được dữ liệu riêng tư của Ứng viên) và BUG_API_002 (link tin mở ra tin khác).</t>
+          <t>•  Dev sửa 20 mã chặn duyệt còn lại ở sheet "Điểm chặn", ưu tiên BUG_API_002 (link tin mở ra tin khác) và Retest_BUG_047 (tin hết hạn vẫn nhận ứng tuyển). BUG_API_003 đã kiểm lại đạt.</t>
         </is>
       </c>
     </row>
@@ -1777,7 +1777,7 @@
     <row r="41" ht="34" customHeight="1">
       <c r="B41" s="18" t="inlineStr">
         <is>
-          <t>•  Cấp tài khoản demo đã kích hoạt (NTD đã xác thực có tin và hồ sơ ứng tuyển như Sanwa / STT 361; Ứng viên Đỗ Minh An) để chạy lại F2–F8 và 40 lỗi Verified cần đăng nhập.</t>
+          <t>•  Chạy lại F2–F8 và 40 lỗi Verified cần đăng nhập bằng các tài khoản demo trong .env (Sanwa = IDOR_NTD1 có tin và hồ sơ ứng tuyển; Ứng viên Đỗ Minh An = CANDIDATE).</t>
         </is>
       </c>
     </row>
@@ -3410,20 +3410,20 @@
           <t>—</t>
         </is>
       </c>
-      <c r="L18" s="27" t="inlineStr">
-        <is>
-          <t>Không xác định</t>
+      <c r="L18" s="28" t="inlineStr">
+        <is>
+          <t>Pass</t>
         </is>
       </c>
       <c r="M18" s="23" t="inlineStr">
         <is>
-          <t>Không xác định (cần tài khoản NTD). Lỗi cần token hợp lệ của tài khoản Nhà tuyển dụng để gọi GET /candidate/applications. Theo quy tắc không đăng nhập và không thử cách khác.</t>
+          <t>GET /candidate/applications bằng token NTD (tài khoản demo EMPLOYER) nay trả HTTP 403, code INVALID_USER_TYPE, "Tài khoản của bạn không có quyền truy cập khu vực này." — đúng kết quả mong đợi. Mới kiểm endpoint ghi trong lỗi gốc; các endpoint /candidate/* khác chưa rà hết.</t>
         </is>
       </c>
       <c r="N18" s="23" t="n"/>
-      <c r="O18" s="24" t="inlineStr">
-        <is>
-          <t>CÒN MỞ</t>
+      <c r="O18" s="28" t="inlineStr">
+        <is>
+          <t>ĐÃ ĐẠT</t>
         </is>
       </c>
     </row>
@@ -4959,20 +4959,20 @@
           <t>—</t>
         </is>
       </c>
-      <c r="L18" s="27" t="inlineStr">
-        <is>
-          <t>Không xác định</t>
+      <c r="L18" s="28" t="inlineStr">
+        <is>
+          <t>Pass</t>
         </is>
       </c>
       <c r="M18" s="23" t="inlineStr">
         <is>
-          <t>Không xác định (cần tài khoản NTD). Lỗi cần token hợp lệ của tài khoản Nhà tuyển dụng để gọi GET /candidate/applications. Theo quy tắc không đăng nhập và không thử cách khác.</t>
+          <t>GET /candidate/applications bằng token NTD (tài khoản demo EMPLOYER) nay trả HTTP 403, code INVALID_USER_TYPE, "Tài khoản của bạn không có quyền truy cập khu vực này." — đúng kết quả mong đợi. Mới kiểm endpoint ghi trong lỗi gốc; các endpoint /candidate/* khác chưa rà hết.</t>
         </is>
       </c>
       <c r="N18" s="23" t="n"/>
-      <c r="O18" s="24" t="inlineStr">
-        <is>
-          <t>CÒN MỞ</t>
+      <c r="O18" s="28" t="inlineStr">
+        <is>
+          <t>ĐÃ ĐẠT</t>
         </is>
       </c>
     </row>
@@ -7501,12 +7501,12 @@
       </c>
       <c r="F8" s="23" t="inlineStr">
         <is>
-          <t>BUG_FUNC_035: CÒN MỞ; BUG_UI_081: CÒN MỞ; BUG_FUNC_017: CÒN MỞ; BUG_UI_082: CÒN MỞ; BUG_API_003: CÒN MỞ</t>
+          <t>BUG_FUNC_035: CÒN MỞ; BUG_UI_081: CÒN MỞ; BUG_FUNC_017: CÒN MỞ; BUG_UI_082: CÒN MỞ; BUG_API_003: ĐÃ ĐẠT</t>
         </is>
       </c>
       <c r="G8" s="23" t="inlineStr">
         <is>
-          <t>BUG_FUNC_035, BUG_UI_081, BUG_FUNC_017, BUG_UI_082, BUG_API_003</t>
+          <t>BUG_FUNC_035, BUG_UI_081, BUG_FUNC_017, BUG_UI_082</t>
         </is>
       </c>
       <c r="H8" s="24" t="inlineStr">

</xml_diff>